<commit_message>
Endocrinology: Excel rebuilt after the final text/answer fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/أزهر دمياط/Endocrinology/Endocrinology_Questions.xlsx
+++ b/أزهر دمياط/Endocrinology/Endocrinology_Questions.xlsx
@@ -35478,7 +35478,7 @@
       </c>
       <c r="I673" t="inlineStr">
         <is>
-          <t>Atrophy of Type II muscle fibers. The answer is</t>
+          <t>Atrophy of Type II muscle fibers.</t>
         </is>
       </c>
       <c r="J673" t="inlineStr">
@@ -35488,7 +35488,7 @@
       </c>
       <c r="R673" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="V673" t="inlineStr">
@@ -44079,7 +44079,7 @@
       </c>
       <c r="I826" t="inlineStr">
         <is>
-          <t>d-Positive family history is less common than in type 11</t>
+          <t>Positive family history is less common than in type 11</t>
         </is>
       </c>
       <c r="J826" t="inlineStr">

</xml_diff>

<commit_message>
Question banks: 169 OCR-garbled stems/options re-read from the page images (in place, answers unchanged)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/أزهر دمياط/Endocrinology/Endocrinology_Questions.xlsx
+++ b/أزهر دمياط/Endocrinology/Endocrinology_Questions.xlsx
@@ -22954,7 +22954,7 @@
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t>HbAIC 5.7-6.4 gm/dl</t>
+          <t>HbA1C 5.7-6.4 gm/dl</t>
         </is>
       </c>
       <c r="G441" t="inlineStr">
@@ -22969,7 +22969,7 @@
       </c>
       <c r="I441" t="inlineStr">
         <is>
-          <t>It is not associated witty increased risk of macrovascular complications</t>
+          <t>It is not associated with increased risk of macrovascular complications</t>
         </is>
       </c>
       <c r="J441" t="inlineStr">
@@ -33534,12 +33534,12 @@
     <row r="641">
       <c r="C641" t="inlineStr">
         <is>
-          <t>Steps in the synthesis of thyro Except: id hormone include all of the following</t>
+          <t>Steps in the synthesis of thyroid hormone include all of the following Except:</t>
         </is>
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>Coupling of iodo-tyrosines,</t>
+          <t>Coupling of iodo-tyrosines.</t>
         </is>
       </c>
       <c r="G641" t="inlineStr">
@@ -33549,12 +33549,12 @@
       </c>
       <c r="H641" t="inlineStr">
         <is>
-          <t>Form active thyroxine b y coupling iodo-tyrosines.</t>
+          <t>Linkage of iodine with tyrosine residues.</t>
         </is>
       </c>
       <c r="I641" t="inlineStr">
         <is>
-          <t>Von Hippel-Lindau syndrome.</t>
+          <t>Oxidation of iodide to iodine.</t>
         </is>
       </c>
       <c r="R641" t="inlineStr">
@@ -33960,7 +33960,7 @@
     <row r="649">
       <c r="C649" t="inlineStr">
         <is>
-          <t>The diagn osis of primary hyperparathyroidism is most strongly su ggested by:</t>
+          <t>The diagnosis of primary hyperparathyroidism is most strongly suggested by:</t>
         </is>
       </c>
       <c r="F649" t="inlineStr">
@@ -33970,22 +33970,22 @@
       </c>
       <c r="G649" t="inlineStr">
         <is>
-          <t>Serum alkaline phosphatase &gt; 120 IU/L,</t>
+          <t>Serum alkaline phosphatase &gt; 120 IU/L.</t>
         </is>
       </c>
       <c r="H649" t="inlineStr">
         <is>
-          <t>Serum calcium &gt; 11 mg/dL,</t>
+          <t>Serum calcium &gt; 11 mg/dL.</t>
         </is>
       </c>
       <c r="I649" t="inlineStr">
         <is>
-          <t>Urinary calcium &lt;100 mg/day</t>
+          <t>Urinary calcium &lt;100 mg/day.</t>
         </is>
       </c>
       <c r="J649" t="inlineStr">
         <is>
-          <t>Parathyroid hormone levels &lt; 5 pmol/L,</t>
+          <t>Parathyroid hormone levels &lt; 5 pmol/L.</t>
         </is>
       </c>
       <c r="R649" t="inlineStr">
@@ -35164,27 +35164,27 @@
     <row r="671">
       <c r="C671" t="inlineStr">
         <is>
-          <t>A 40-year-old male undergoes an aed ene r '. thyroidectomy for follicular carcinoma of develops circum-oral numbness, followed by laryngospasm, and then a generalized seizure. Of the following, which is the first priority 'or ex. operative site.</t>
+          <t>A 40-year-old male undergoes an apparently uneventful total thyroidectomy for follicular carcinoma of the thyroid. 48 hours later he develops circum-oral numbness, followed by laryngospasm, and then has a generalized seizure. Of the following, which is the first priority?</t>
         </is>
       </c>
       <c r="F671" t="inlineStr">
         <is>
-          <t>Proceed to OR for exploration of the of</t>
+          <t>Proceed to OR for exploration of the operative site.</t>
         </is>
       </c>
       <c r="G671" t="inlineStr">
         <is>
-          <t>Administer 25 ml of 10 calcium g 10% calet Jucon</t>
+          <t>Administer 25 ml of 10% calcium gluconate intravenously.</t>
         </is>
       </c>
       <c r="H671" t="inlineStr">
         <is>
-          <t>Obtain a serum 1; and administer intravenous. jagnesium measurement chlonde STAT.</t>
+          <t>Obtain a serum magnesium measurement and administer intravenous magnesium chloride STAT.</t>
         </is>
       </c>
       <c r="I671" t="inlineStr">
         <is>
-          <t>Obtain a CT scan of the head to ev</t>
+          <t>Obtain a CT scan of the head to evaluate the possibility of brain metastases.</t>
         </is>
       </c>
       <c r="R671" t="inlineStr">

</xml_diff>